<commit_message>
feat: update labor book template and service to match report format requirements and default null values
</commit_message>
<xml_diff>
--- a/backend/src/main/resources/hr/templates/labor-book-template.xlsx
+++ b/backend/src/main/resources/hr/templates/labor-book-template.xlsx
@@ -670,32 +670,32 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DOANH NGHIỆP: CÔNG TY CỔ PHẦN PHÂN BÓN VÀ HÓA CHẤT CẦN THƠ</t>
+          <t>DOANH NGHIỆP……………………….</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mã số thuế: 1800156719</t>
+          <t>Mã số thuế: ………………………………………..</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Địa chỉ: Khu vực Thới Thạnh, Phường Thới An, Quận Ô Môn, Thành phố Cần Thơ</t>
+          <t>Địa chỉ: ………………………………………..</t>
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="32.25" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>SỔ QUẢN LÝ LAO ĐỘNG</t>
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>STT</t>
@@ -819,7 +819,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="123.75" customHeight="1">
       <c r="A6" s="10" t="n"/>
       <c r="B6" s="10" t="n"/>
       <c r="C6" s="10" t="n"/>
@@ -859,7 +859,7 @@
       <c r="Y6" s="10" t="n"/>
       <c r="Z6" s="10" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="18" customHeight="1">
       <c r="A7" s="11" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
feat: update labor book export service to include address, position, and leave days in template
</commit_message>
<xml_diff>
--- a/backend/src/main/resources/hr/templates/labor-book-template.xlsx
+++ b/backend/src/main/resources/hr/templates/labor-book-template.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -221,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -273,6 +272,30 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -643,22 +666,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.42578125" customWidth="1" min="1" max="1"/>
-    <col width="30.140625" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="9.28515625" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="9.42578125" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
     <col width="16.7109375" customWidth="1" min="8" max="8"/>
-    <col width="14.140625" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="6.42578125" customWidth="1" min="11" max="11"/>
-    <col width="23.5703125" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="13.85546875" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="14.85546875" customWidth="1" min="18" max="18"/>
     <col width="7.28515625" customWidth="1" min="19" max="19"/>
-    <col width="8.5703125" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
     <col width="9.140625" customWidth="1" min="21" max="21"/>
     <col width="10" customWidth="1" min="22" max="22"/>
     <col width="11.42578125" customWidth="1" min="23" max="23"/>
@@ -859,77 +882,77 @@
       <c r="Y6" s="10" t="n"/>
       <c r="Z6" s="10" t="n"/>
     </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="11" t="n">
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>A268</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr">
         <is>
           <t>Nguyễn Công Huân</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>Nam</t>
         </is>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="23" t="n">
         <v>31483</v>
       </c>
-      <c r="F7" s="15" t="inlineStr">
+      <c r="F7" s="24" t="inlineStr">
         <is>
           <t>Việt Nam</t>
         </is>
       </c>
-      <c r="G7" s="11" t="n"/>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="G7" s="20" t="n"/>
+      <c r="H7" s="25" t="inlineStr">
         <is>
           <t>092086007417</t>
         </is>
       </c>
-      <c r="I7" s="17" t="inlineStr">
+      <c r="I7" s="22" t="inlineStr">
         <is>
           <t>Thạc sĩ</t>
         </is>
       </c>
-      <c r="J7" s="11" t="n"/>
-      <c r="K7" s="15" t="n"/>
-      <c r="L7" s="17" t="inlineStr">
+      <c r="J7" s="20" t="n"/>
+      <c r="K7" s="24" t="n"/>
+      <c r="L7" s="22" t="inlineStr">
         <is>
           <t>Không xác định</t>
         </is>
       </c>
-      <c r="M7" s="14" t="n">
+      <c r="M7" s="23" t="n">
         <v>41379</v>
       </c>
-      <c r="N7" s="14" t="n">
+      <c r="N7" s="23" t="n">
         <v>41379</v>
       </c>
-      <c r="O7" s="14" t="n">
+      <c r="O7" s="23" t="n">
         <v>41379</v>
       </c>
-      <c r="P7" s="14" t="n">
+      <c r="P7" s="23" t="n">
         <v>41379</v>
       </c>
-      <c r="Q7" s="18" t="n">
+      <c r="Q7" s="26" t="n">
         <v>26000000</v>
       </c>
-      <c r="R7" s="18" t="n">
+      <c r="R7" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="S7" s="15" t="n"/>
-      <c r="T7" s="19" t="n"/>
-      <c r="U7" s="19" t="n"/>
-      <c r="V7" s="15" t="n"/>
-      <c r="W7" s="15" t="n"/>
-      <c r="X7" s="15" t="n"/>
-      <c r="Y7" s="15" t="n"/>
-      <c r="Z7" s="15" t="n"/>
+      <c r="S7" s="24" t="n"/>
+      <c r="T7" s="24" t="n"/>
+      <c r="U7" s="27" t="n"/>
+      <c r="V7" s="24" t="n"/>
+      <c r="W7" s="24" t="n"/>
+      <c r="X7" s="24" t="n"/>
+      <c r="Y7" s="24" t="n"/>
+      <c r="Z7" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="28">

</xml_diff>